<commit_message>
Add teacher task management & offline mocks
Added teacher task managment page
Added student answer form
Deleted "back" button
Updated frontend/api.xlsx
</commit_message>
<xml_diff>
--- a/frontend/api.xlsx
+++ b/frontend/api.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="50">
   <si>
     <t>Endpoint</t>
   </si>
@@ -102,6 +102,81 @@
   </si>
   <si>
     <t>^ смотри Bearer JWT</t>
+  </si>
+  <si>
+    <t>Discription</t>
+  </si>
+  <si>
+    <t>вход в систему для обоих ролей</t>
+  </si>
+  <si>
+    <t>кто я?</t>
+  </si>
+  <si>
+    <t>детальная информация о задании для студента</t>
+  </si>
+  <si>
+    <t>отправка ответа на задание студентом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">список отчётов для преподавателя
+</t>
+  </si>
+  <si>
+    <t>обновление статуса и оценки отчёта</t>
+  </si>
+  <si>
+    <t xml:space="preserve">список заданий для студента
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">детальная информация об отчёте
+</t>
+  </si>
+  <si>
+    <t>/api/teacher/tasks</t>
+  </si>
+  <si>
+    <t>title, description, group_number, subject_name</t>
+  </si>
+  <si>
+    <t>/api/teacher/tasks/{task_id}</t>
+  </si>
+  <si>
+    <t>редактирование задания преподавателем</t>
+  </si>
+  <si>
+    <t>/api/teacher/tasks/{task_id}/delete</t>
+  </si>
+  <si>
+    <t>удаление задания преподавателем</t>
+  </si>
+  <si>
+    <t>получение всех заданий преподавателем</t>
+  </si>
+  <si>
+    <t>[{ task_id, title, subject_name, group_number, description }]</t>
+  </si>
+  <si>
+    <t>получение конкретного задания преподавателем</t>
+  </si>
+  <si>
+    <t>{ task_id, title, subject_name, group_number, description }</t>
+  </si>
+  <si>
+    <t>добавление задания преподавателем</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Both</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Teacher</t>
   </si>
 </sst>
 </file>
@@ -140,7 +215,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -163,14 +238,85 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -451,193 +597,361 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="97.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="4"/>
+    <col min="2" max="2" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="97.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="56.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="G1" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="19.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G2" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G3" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G6" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G7" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="G8" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
+      <c r="G9" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="C12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
     </row>
   </sheetData>
+  <sortState ref="A1:G14">
+    <sortCondition ref="A2:A14"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>